<commit_message>
feat: actualizar archivos de presentación y codificación total
</commit_message>
<xml_diff>
--- a/_docs/trim_02/Contextualizacion Proyecto/Porcentaje de codificacion total.xlsx
+++ b/_docs/trim_02/Contextualizacion Proyecto/Porcentaje de codificacion total.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\AXXION_SYSTEM_\_docs\trim_02\Contextualizacion Proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49793A34-4E1D-4777-9417-5286377835EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F05090F-897D-4FD1-A0A6-7EABB1629528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{6CD96AF1-C494-414E-A4C6-796DD518F531}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6CD96AF1-C494-414E-A4C6-796DD518F531}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="59">
   <si>
     <t>RF</t>
   </si>
@@ -191,27 +191,9 @@
     <t>Actualizar historial de mantenimiento</t>
   </si>
   <si>
-    <t>Configurar alertas por activo (ej. vencimiento de garantía, próxima revisión, devolución de alquiler)</t>
-  </si>
-  <si>
     <t>Consultar todas las alertas configuradas</t>
   </si>
   <si>
-    <t>Consultar alerta</t>
-  </si>
-  <si>
-    <t>Actualizar alerta</t>
-  </si>
-  <si>
-    <t>Eliminar alerta (cambiar de estado)</t>
-  </si>
-  <si>
-    <t>Generar notificación de alerta</t>
-  </si>
-  <si>
-    <t>Consultar historial de notificaciones</t>
-  </si>
-  <si>
     <t>Generar reporte de activos tecnológicos</t>
   </si>
   <si>
@@ -224,13 +206,13 @@
     <t>Generar reporte de usuarios</t>
   </si>
   <si>
-    <t>Exportar reportes (PDF, Excel, CSV)</t>
-  </si>
-  <si>
     <t>Porcentaje</t>
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Exportar reportes (Excel)</t>
   </si>
 </sst>
 </file>
@@ -274,7 +256,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -341,6 +323,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -392,7 +380,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -427,6 +415,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -773,11 +762,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EE07042-B933-4627-BAC2-B36C8B2EB8A1}">
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="79.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="87.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -805,13 +794,13 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -822,13 +811,13 @@
         <v>5</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -842,7 +831,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="I4" s="15">
         <v>174</v>
@@ -858,25 +847,19 @@
       <c r="B5" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>64</v>
-      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="9"/>
       <c r="G5" s="17">
         <f>I5/I4</f>
-        <v>0.79885057471264365</v>
+        <v>0.78735632183908044</v>
       </c>
       <c r="I5" s="15">
-        <f>COUNTIF(C2:E59,"x")</f>
-        <v>139</v>
+        <f>COUNTIF(C2:E53,"x")</f>
+        <v>137</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -887,12 +870,14 @@
         <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
@@ -902,13 +887,13 @@
         <v>9</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -918,12 +903,8 @@
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>64</v>
-      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -933,15 +914,9 @@
       <c r="B9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>64</v>
-      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="9"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
@@ -951,13 +926,13 @@
         <v>12</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -968,13 +943,13 @@
         <v>13</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -985,13 +960,13 @@
         <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -1002,13 +977,13 @@
         <v>15</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -1019,13 +994,13 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -1036,13 +1011,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -1053,13 +1028,13 @@
         <v>19</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -1070,13 +1045,13 @@
         <v>20</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -1087,13 +1062,13 @@
         <v>21</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -1104,13 +1079,13 @@
         <v>22</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -1121,13 +1096,13 @@
         <v>23</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -1138,13 +1113,13 @@
         <v>24</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1155,13 +1130,13 @@
         <v>25</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -1172,13 +1147,13 @@
         <v>26</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -1189,13 +1164,13 @@
         <v>27</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1206,13 +1181,13 @@
         <v>28</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -1223,13 +1198,13 @@
         <v>29</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -1240,13 +1215,13 @@
         <v>30</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -1257,13 +1232,13 @@
         <v>31</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -1274,13 +1249,13 @@
         <v>32</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1291,12 +1266,14 @@
         <v>33</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E30" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="14">
@@ -1306,12 +1283,14 @@
         <v>34</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E31" s="9"/>
+        <v>57</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="5">
@@ -1321,12 +1300,14 @@
         <v>35</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E32" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="14">
@@ -1336,12 +1317,14 @@
         <v>36</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E33" s="9"/>
+        <v>57</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="5">
@@ -1351,12 +1334,14 @@
         <v>37</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E34" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="14">
@@ -1366,12 +1351,14 @@
         <v>38</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E35" s="9"/>
+        <v>57</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="5">
@@ -1381,12 +1368,14 @@
         <v>39</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E36" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="14">
@@ -1396,12 +1385,14 @@
         <v>40</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E37" s="9"/>
+        <v>57</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="5">
@@ -1411,12 +1402,14 @@
         <v>41</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E38" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="14">
@@ -1426,12 +1419,14 @@
         <v>42</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E39" s="9"/>
+        <v>57</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="5">
@@ -1441,13 +1436,13 @@
         <v>43</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -1458,13 +1453,13 @@
         <v>44</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -1475,13 +1470,13 @@
         <v>45</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -1492,13 +1487,13 @@
         <v>46</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -1509,13 +1504,13 @@
         <v>47</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
@@ -1526,7 +1521,7 @@
         <v>48</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D45" s="10"/>
       <c r="E45" s="9"/>
@@ -1539,7 +1534,7 @@
         <v>49</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
@@ -1556,189 +1551,113 @@
       <c r="E47" s="9"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="5">
-        <v>47</v>
-      </c>
-      <c r="B48" s="1" t="s">
+      <c r="A48" s="14">
+        <v>48</v>
+      </c>
+      <c r="B48" s="18" t="s">
         <v>51</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="14">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>52</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="5">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>53</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="14">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B51" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="C51" s="11"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="9"/>
+      <c r="C51" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="5">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C52" s="11"/>
-      <c r="D52" s="1"/>
-      <c r="E52" s="1"/>
+      <c r="C52" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="14">
-        <v>52</v>
-      </c>
-      <c r="B53" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C53" s="11"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="9"/>
+      <c r="B53" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C53" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="5">
-        <v>53</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C54" s="11"/>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="14">
-        <v>54</v>
-      </c>
-      <c r="B55" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E55" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="5">
-        <v>55</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C56" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A57" s="14">
-        <v>56</v>
-      </c>
-      <c r="B57" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="C57" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D57" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E57" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A58" s="5">
-        <v>57</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C58" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A59" s="14">
-        <v>58</v>
-      </c>
-      <c r="B59" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="C59" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D59" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E59" s="9"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
+      <c r="A54" s="4"/>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>

<commit_message>
feat: Update project documentation and add automation tests
- Updated Excel files for project coding percentage and test cases.
- Added new presentation file for project context.
- Removed obsolete delete.txt file.
- Introduced Gradle build configuration for automation tests.
- Added .gitignore to exclude unnecessary files from version control.
- Created initial Gradle wrapper files for project setup.
- Implemented test feature files for adding, editing, and consulting categories and subcategories.
- Updated backend dependencies and security configurations.
- Enhanced frontend views for better user experience and accessibility.
</commit_message>
<xml_diff>
--- a/_docs/trim_02/Contextualizacion Proyecto/Porcentaje de codificacion total.xlsx
+++ b/_docs/trim_02/Contextualizacion Proyecto/Porcentaje de codificacion total.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\AXXION_SYSTEM_\_docs\trim_02\Contextualizacion Proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F05090F-897D-4FD1-A0A6-7EABB1629528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD3950EB-437E-4E54-BDEC-C06C3827586F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6CD96AF1-C494-414E-A4C6-796DD518F531}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{6CD96AF1-C494-414E-A4C6-796DD518F531}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="52">
   <si>
     <t>RF</t>
   </si>
@@ -56,24 +56,12 @@
     <t>Cerrar Sesión</t>
   </si>
   <si>
-    <t>Recuperar contraseña</t>
-  </si>
-  <si>
-    <t>Registrar roles</t>
-  </si>
-  <si>
     <t>Consultar todos los roles</t>
   </si>
   <si>
     <t>Consultar un rol</t>
   </si>
   <si>
-    <t>Actualizar rol</t>
-  </si>
-  <si>
-    <t>Eliminar rol (Cambiar de Estado)</t>
-  </si>
-  <si>
     <t>Registrar usuarios</t>
   </si>
   <si>
@@ -86,9 +74,6 @@
     <t>Actualizar usuario</t>
   </si>
   <si>
-    <t>Eliminar usuario (Cambiar de Estado)</t>
-  </si>
-  <si>
     <t>#</t>
   </si>
   <si>
@@ -104,9 +89,6 @@
     <t>Actualizar categoría</t>
   </si>
   <si>
-    <t>Eliminar categoría (cambiar de estado)</t>
-  </si>
-  <si>
     <t>Registrar subcategorías</t>
   </si>
   <si>
@@ -119,9 +101,6 @@
     <t>Actualizar subcategoría</t>
   </si>
   <si>
-    <t>Eliminar subcategoría (cambiar de estado)</t>
-  </si>
-  <si>
     <t>Registrar activos tecnológicos</t>
   </si>
   <si>
@@ -134,9 +113,6 @@
     <t>Actualizar activo</t>
   </si>
   <si>
-    <t>Eliminar activo (cambiar de estado)</t>
-  </si>
-  <si>
     <t>Registrar solicitud de alquiler</t>
   </si>
   <si>
@@ -149,9 +125,6 @@
     <t>Actualizar solicitud de alquiler</t>
   </si>
   <si>
-    <t>Cancelar solicitud de alquiler (cambiar de estado)</t>
-  </si>
-  <si>
     <t>Registrar contrato de alquiler</t>
   </si>
   <si>
@@ -164,9 +137,6 @@
     <t>Actualizar contrato</t>
   </si>
   <si>
-    <t>Finalizar contrato (cambiar de estado)</t>
-  </si>
-  <si>
     <t>Registrar solicitud de mantenimiento</t>
   </si>
   <si>
@@ -179,18 +149,6 @@
     <t>Actualizar solicitud de mantenimiento</t>
   </si>
   <si>
-    <t>Cancelar solicitud de mantenimiento (cambiar de estado)</t>
-  </si>
-  <si>
-    <t>Registrar historial de mantenimiento</t>
-  </si>
-  <si>
-    <t>Consultar historial de mantenimiento por activo</t>
-  </si>
-  <si>
-    <t>Actualizar historial de mantenimiento</t>
-  </si>
-  <si>
     <t>Consultar todas las alertas configuradas</t>
   </si>
   <si>
@@ -213,6 +171,27 @@
   </si>
   <si>
     <t>Exportar reportes (Excel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eliminar categoría </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eliminar usuario </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eliminar subcategoría </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancelar solicitud de alquiler </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eliminar activo </t>
+  </si>
+  <si>
+    <t>Finalizar contrato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancelar solicitud de mantenimiento </t>
   </si>
 </sst>
 </file>
@@ -380,7 +359,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -411,9 +390,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
@@ -762,16 +738,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EE07042-B933-4627-BAC2-B36C8B2EB8A1}">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="87.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -786,7 +762,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -794,16 +770,16 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="14">
         <v>2</v>
       </c>
@@ -811,58 +787,64 @@
         <v>5</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
+      <c r="C4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="G4" s="1" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="I4" s="15">
-        <v>174</v>
-      </c>
-      <c r="J4" s="15">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="14">
         <v>4</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="9"/>
-      <c r="G5" s="17">
+      <c r="C5" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" s="16">
         <f>I5/I4</f>
-        <v>0.78735632183908044</v>
+        <v>1</v>
       </c>
       <c r="I5" s="15">
-        <f>COUNTIF(C2:E53,"x")</f>
-        <v>137</v>
-      </c>
-      <c r="J5" s="16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+        <f>COUNTIF(C2:E46,"x")</f>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -870,16 +852,16 @@
         <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
         <v>6</v>
       </c>
@@ -887,55 +869,67 @@
         <v>9</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>8</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>10</v>
       </c>
@@ -943,33 +937,33 @@
         <v>13</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>57</v>
+      <c r="C12" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>12</v>
       </c>
@@ -977,64 +971,64 @@
         <v>15</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>57</v>
+      <c r="C14" s="11" t="s">
+        <v>43</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>14</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -1042,16 +1036,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -1059,16 +1053,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -1076,16 +1070,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -1093,16 +1087,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -1110,16 +1104,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1127,16 +1121,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -1144,16 +1138,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -1161,16 +1155,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1178,16 +1172,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -1195,16 +1189,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -1212,16 +1206,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -1229,16 +1223,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -1246,16 +1240,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1263,16 +1257,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -1280,16 +1274,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -1297,16 +1291,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -1314,16 +1308,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -1331,16 +1325,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -1348,16 +1342,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
@@ -1365,16 +1359,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -1382,16 +1376,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -1399,16 +1393,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -1416,16 +1410,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -1433,231 +1427,126 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="14">
         <v>40</v>
       </c>
-      <c r="B41" s="12" t="s">
-        <v>44</v>
+      <c r="B41" s="17" t="s">
+        <v>37</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="5">
         <v>41</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>45</v>
+      <c r="B42" s="12" t="s">
+        <v>38</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="14">
         <v>42</v>
       </c>
-      <c r="B43" s="12" t="s">
-        <v>46</v>
+      <c r="B43" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E43" s="9" t="s">
-        <v>57</v>
+        <v>43</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="5">
         <v>43</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>47</v>
+      <c r="B44" s="12" t="s">
+        <v>40</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="14">
         <v>44</v>
       </c>
-      <c r="B45" s="12" t="s">
-        <v>48</v>
+      <c r="B45" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D45" s="10"/>
-      <c r="E45" s="9"/>
+        <v>43</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="5">
         <v>45</v>
       </c>
-      <c r="B46" s="1" t="s">
-        <v>49</v>
+      <c r="B46" s="13" t="s">
+        <v>44</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="14">
-        <v>46</v>
-      </c>
-      <c r="B47" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C47" s="11"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="9"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="14">
-        <v>48</v>
-      </c>
-      <c r="B48" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="C48" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E48" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="14">
-        <v>52</v>
-      </c>
-      <c r="B49" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="5">
-        <v>53</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C50" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51" s="14">
-        <v>54</v>
-      </c>
-      <c r="B51" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C51" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D51" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A52" s="5">
-        <v>55</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C52" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="14">
-        <v>56</v>
-      </c>
-      <c r="B53" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C53" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="D53" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E53" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="4"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>